<commit_message>
Petite Cup 57 (S4 Round 7): Jake wins PCDJ #56, 39 players
</commit_message>
<xml_diff>
--- a/Petite Cups 56-60.xlsx
+++ b/Petite Cups 56-60.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:D59"/>
+  <dimension ref="A2:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -422,6 +422,11 @@
           <t>Petite Cup 56</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Petite Cup 57</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -429,6 +434,11 @@
           <t>Maps: PCDJ #55 - Tori by [CSC] PlusMicron + PCDJ #55 - Inline by felix</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Maps: PCDJ #56 - Mountain Coppice by redal + PCDJ #56 Tiny Radiant Halls by sanhe</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -447,6 +457,26 @@
         </is>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -464,6 +494,17 @@
       <c r="C6" t="n">
         <v>19.54192</v>
       </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Jake</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>20.12153</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -480,6 +521,22 @@
       <c r="D7" t="n">
         <v>14</v>
       </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[KBW]microways</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -496,6 +553,20 @@
       <c r="D8" t="n">
         <v>13</v>
       </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Sterben</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>19.85596</v>
+      </c>
+      <c r="J8" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -514,6 +585,20 @@
       <c r="D9" t="n">
         <v>12</v>
       </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>[MMM]LKat</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>20.37223</v>
+      </c>
+      <c r="J9" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -532,6 +617,20 @@
       <c r="D10" t="n">
         <v>11</v>
       </c>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>19.85143</v>
+      </c>
+      <c r="J10" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -548,6 +647,20 @@
       <c r="D11" t="n">
         <v>10</v>
       </c>
+      <c r="G11" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ZOMAN</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>20.45766</v>
+      </c>
+      <c r="J11" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -564,6 +677,20 @@
       <c r="D12" t="n">
         <v>10</v>
       </c>
+      <c r="G12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>[CSC]Tommygaming</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>19.82093</v>
+      </c>
+      <c r="J12" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -580,6 +707,20 @@
       <c r="D13" t="n">
         <v>9</v>
       </c>
+      <c r="G13" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>19.91285</v>
+      </c>
+      <c r="J13" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -596,6 +737,20 @@
       <c r="D14" t="n">
         <v>9</v>
       </c>
+      <c r="G14" t="n">
+        <v>9</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>[WASH] Quickracer10</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>20.50894</v>
+      </c>
+      <c r="J14" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -612,6 +767,20 @@
       <c r="D15" t="n">
         <v>8</v>
       </c>
+      <c r="G15" t="n">
+        <v>10</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>[CSC]AndMe18</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>20.56719</v>
+      </c>
+      <c r="J15" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -628,6 +797,20 @@
       <c r="D16" t="n">
         <v>8</v>
       </c>
+      <c r="G16" t="n">
+        <v>11</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>[CSC] PlusMicron</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>19.95048</v>
+      </c>
+      <c r="J16" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -644,6 +827,20 @@
       <c r="D17" t="n">
         <v>7</v>
       </c>
+      <c r="G17" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[MMM]Victor</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>19.99004</v>
+      </c>
+      <c r="J17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -662,6 +859,20 @@
       <c r="D18" t="n">
         <v>7</v>
       </c>
+      <c r="G18" t="n">
+        <v>13</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>20.99734</v>
+      </c>
+      <c r="J18" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -678,6 +889,22 @@
       <c r="D19" t="n">
         <v>6</v>
       </c>
+      <c r="G19" t="n">
+        <v>14</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Mμ</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -694,6 +921,20 @@
       <c r="D20" t="n">
         <v>6</v>
       </c>
+      <c r="G20" t="n">
+        <v>15</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>20.10806</v>
+      </c>
+      <c r="J20" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -710,6 +951,20 @@
       <c r="D21" t="n">
         <v>6</v>
       </c>
+      <c r="G21" t="n">
+        <v>16</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Gimpel</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>20.15303</v>
+      </c>
+      <c r="J21" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -726,6 +981,20 @@
       <c r="D22" t="n">
         <v>5</v>
       </c>
+      <c r="G22" t="n">
+        <v>17</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>[CSC] variableferret</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>20.1722</v>
+      </c>
+      <c r="J22" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -742,6 +1011,22 @@
       <c r="D23" t="n">
         <v>5</v>
       </c>
+      <c r="G23" t="n">
+        <v>18</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>MALIYO</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -758,6 +1043,22 @@
       <c r="D24" t="n">
         <v>5</v>
       </c>
+      <c r="G24" t="n">
+        <v>18</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -774,6 +1075,22 @@
       <c r="D25" t="n">
         <v>4</v>
       </c>
+      <c r="G25" t="n">
+        <v>18</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>jandje</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -790,6 +1107,20 @@
       <c r="D26" t="n">
         <v>4</v>
       </c>
+      <c r="G26" t="n">
+        <v>21</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>[MMM]Kreeeeee</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>20.20749</v>
+      </c>
+      <c r="J26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -808,6 +1139,20 @@
       <c r="D27" t="n">
         <v>4</v>
       </c>
+      <c r="G27" t="n">
+        <v>22</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>cookie</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>20.2574</v>
+      </c>
+      <c r="J27" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -824,6 +1169,20 @@
       <c r="D28" t="n">
         <v>3</v>
       </c>
+      <c r="G28" t="n">
+        <v>23</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>wokonbike</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>20.42944</v>
+      </c>
+      <c r="J28" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -842,6 +1201,22 @@
       <c r="D29" t="n">
         <v>3</v>
       </c>
+      <c r="G29" t="n">
+        <v>24</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Jorts</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -860,6 +1235,22 @@
       <c r="D30" t="n">
         <v>3</v>
       </c>
+      <c r="G30" t="n">
+        <v>24</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>[CSC]IronDragon111000</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -876,6 +1267,22 @@
       <c r="D31" t="n">
         <v>2</v>
       </c>
+      <c r="G31" t="n">
+        <v>24</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>[SLOW]Zeus</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -894,6 +1301,22 @@
       <c r="D32" t="n">
         <v>2</v>
       </c>
+      <c r="G32" t="n">
+        <v>24</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>gilgool</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -912,6 +1335,20 @@
       <c r="D33" t="n">
         <v>2</v>
       </c>
+      <c r="G33" t="n">
+        <v>28</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>20.4619</v>
+      </c>
+      <c r="J33" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -930,6 +1367,20 @@
       <c r="D34" t="n">
         <v>1</v>
       </c>
+      <c r="G34" t="n">
+        <v>29</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>20.5721</v>
+      </c>
+      <c r="J34" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -948,6 +1399,20 @@
       <c r="D35" t="n">
         <v>1</v>
       </c>
+      <c r="G35" t="n">
+        <v>30</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>ActuallyRuben</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>21.00119</v>
+      </c>
+      <c r="J35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -966,6 +1431,22 @@
       <c r="D36" t="n">
         <v>1</v>
       </c>
+      <c r="G36" t="n">
+        <v>31</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>DaimyoN</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -984,6 +1465,22 @@
       <c r="D37" t="n">
         <v>1</v>
       </c>
+      <c r="G37" t="n">
+        <v>31</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Shinikage221</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1002,13 +1499,129 @@
       <c r="D38" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
+      <c r="G38" t="n">
+        <v>31</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>[CSC]K410K3N</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="G39" t="n">
+        <v>31</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>linx200</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="G40" t="n">
+        <v>31</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>meganuke22</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="G41" t="n">
+        <v>31</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>󠀡󠀡᠌ ⁧⁧Thalli</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="G42" t="n">
+        <v>37</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>AndrewIF</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="G43" t="n">
+        <v>38</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="G44" t="n">
+        <v>38</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>rtube</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
+    </row>
     <row r="45"/>
     <row r="46"/>
     <row r="47"/>

</xml_diff>